<commit_message>
Daily Stock Data & Scanner Update - 2026-07-19 16:16 UTC
</commit_message>
<xml_diff>
--- a/Output/MACD Normal Divergences_19 Jul 2026.xlsx
+++ b/Output/MACD Normal Divergences_19 Jul 2026.xlsx
@@ -881,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -949,7 +949,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>21STCENMGM</t>
+          <t>ABDL</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -962,7 +962,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Bullish ND</t>
+          <t>Bearish ND</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -972,7 +972,157 @@
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AABDL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ABBOTINDIA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bullish ND</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AABBOTINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>21STCENMGM</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Bullish ND</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3A21STCENMGM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ABAN</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Bullish ND</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AABAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>A2ZINFRA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Bullish ND</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AA2ZINFRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ABCAPITAL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Bearish ND</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AABCAPITAL</t>
         </is>
       </c>
     </row>
@@ -987,7 +1137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1055,20 +1205,152 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>No scanner alerts detected for this interval</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
+          <t>AAKASH</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Bullish ND</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AAAKASH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AAVAS</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Bullish ND</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AAAVAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ABMINTLLTD</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Bullish ND</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AABMINTLLTD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ACL</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Bullish ND</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AACL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ADANIPORTS</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Divergence Alert</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Bearish ND</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://in.tradingview.com/chart/LqUZraZ9/?symbol=NSE%3AADANIPORTS</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>